<commit_message>
Add meeting and sprint documentation
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_1_Backlog.xlsx
+++ b/documentation/scrum/Sprint_1_Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="136" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E8814E4-A2C2-4DA4-BD84-172996848254}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BBBB7FE-883F-49C4-965E-9F50DA3B4476}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="116">
   <si>
     <t>CIS4014-N Interactive Visualisation – Group 4 | Sprint 1 – Week 01</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>Week 01</t>
-  </si>
-  <si>
     <t>Sprint Goal</t>
   </si>
   <si>
@@ -209,9 +206,6 @@
     <t>Shared Trello board</t>
   </si>
   <si>
-    <t>Day 1–2</t>
-  </si>
-  <si>
     <t>Create GitHub repository and invite team</t>
   </si>
   <si>
@@ -254,9 +248,6 @@
     <t>Next sprint priorities</t>
   </si>
   <si>
-    <t>End of Week 01</t>
-  </si>
-  <si>
     <t>Meeting_01.docx</t>
   </si>
   <si>
@@ -276,9 +267,6 @@
   </si>
   <si>
     <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/README_STRUCTURE.md</t>
-  </si>
-  <si>
-    <t>Uploaded to documentation/meetings to github</t>
   </si>
   <si>
     <t>Coffe Shop Sales Dataset</t>
@@ -413,6 +401,33 @@
   </si>
   <si>
     <t>S1-20</t>
+  </si>
+  <si>
+    <t>Week 01(20 September 2026 – 26 September 2026)</t>
+  </si>
+  <si>
+    <t>20 September 2026   (Day 0)</t>
+  </si>
+  <si>
+    <t>21 September 2026   (Day 1)</t>
+  </si>
+  <si>
+    <t>22 September 2026   (Day 2)</t>
+  </si>
+  <si>
+    <t>23 September 2026   (Day 3)</t>
+  </si>
+  <si>
+    <t>24 September 2026   (Day 4)</t>
+  </si>
+  <si>
+    <t>25 September 2026   (Day 5)</t>
+  </si>
+  <si>
+    <t>26 September 2026   (Day 6)</t>
+  </si>
+  <si>
+    <t>Uploaded to "documentation/meeting" to github</t>
   </si>
 </sst>
 </file>
@@ -507,7 +522,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -551,6 +566,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -591,8 +609,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Sprint1Tasks" displayName="Sprint1Tasks" ref="A11:I29" headerRowDxfId="1">
-  <autoFilter ref="A11:I29" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Sprint1Tasks" displayName="Sprint1Tasks" ref="A11:I31" headerRowDxfId="1">
+  <autoFilter ref="A11:I31" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Task ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Sprint Task"/>
@@ -897,12 +915,12 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="2" max="2" width="41.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="42" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="7" max="7" width="17.08984375" customWidth="1"/>
     <col min="8" max="8" width="85.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="101.36328125" style="7" customWidth="1"/>
   </cols>
@@ -931,575 +949,575 @@
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
+      <c r="B4" s="17" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.5">
       <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="58">
       <c r="A7" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="43.5">
       <c r="A8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="29">
       <c r="A9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="14" customFormat="1">
       <c r="A11" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="D11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="E11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="F11" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="G11" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="H11" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="I11" s="13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="29">
+      <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="B12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="31" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="I13" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="29">
       <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>4</v>
+      <c r="G14" s="7" t="s">
+        <v>108</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="29">
       <c r="A15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="G15" s="2" t="s">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="29">
       <c r="A16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="G16" s="2" t="s">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="29">
       <c r="A17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="G17" s="2" t="s">
-        <v>4</v>
+        <v>109</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="29">
       <c r="A18" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="G18" s="2" t="s">
-        <v>4</v>
+        <v>109</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="29">
       <c r="A19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="G19" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="29">
+      <c r="A20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I20" s="6"/>
+    </row>
+    <row r="21" spans="1:9" ht="29">
+      <c r="A21" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I21" s="6"/>
+    </row>
+    <row r="22" spans="1:9" ht="29">
+      <c r="A22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="I22" s="6"/>
+    </row>
+    <row r="23" spans="1:9" ht="29">
+      <c r="A23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="29">
+      <c r="A24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="29">
+      <c r="A25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H25" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="I20" s="6"/>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="I21" s="6"/>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="I22" s="6"/>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="33" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="29">
+      <c r="A27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="B27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E26" s="2" t="s">
+      <c r="E27" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="29">
+      <c r="A28" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="29">
+      <c r="A29" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="A27" s="2" t="s">
+      <c r="B29" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I27" s="11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="A28" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="I28" s="11" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="G29" s="2" t="s">
-        <v>73</v>
+        <v>114</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>